<commit_message>
Update Fossil Replenishment and Cluster data files
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/Cluster.xlsx
+++ b/data/input/Fossil Replenishment/Cluster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7F7E2068-6C25-4538-9CCF-4A3817287E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017CE957-FEAA-456C-BD6A-B529328FB879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F651F294-041D-4851-877B-E12544EA1683}"/>
   </bookViews>
@@ -469,6 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44A6BF5F-698F-4409-BCD5-2245EEFFB050}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -480,7 +481,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -504,7 +505,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -512,7 +513,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -520,7 +521,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -528,7 +529,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -536,7 +537,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -544,7 +545,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -552,7 +553,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -560,7 +561,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -568,7 +569,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -584,7 +585,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -600,7 +601,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -624,7 +625,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -633,6 +634,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B20" xr:uid="{44A6BF5F-698F-4409-BCD5-2245EEFFB050}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="BOM"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>